<commit_message>
Add Exercises module and update QA documentation
</commit_message>
<xml_diff>
--- a/02_Yetkisiz_Kullanıcı_Kayıt_ve_Giriş/2 - UA - SISU.xlsx
+++ b/02_Yetkisiz_Kullanıcı_Kayıt_ve_Giriş/2 - UA - SISU.xlsx
@@ -5,19 +5,19 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bovay\Desktop\¨¨¨¨¨¨\PROJECTS\CV TASLAK\POWER PULSE - PROJE\PLANLAMA\02. YETKİSİZ KULLANICI - KAYIT VE GİRİŞ\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bovay\Desktop\¨¨¨¨¨¨\PROJECTS\CV TASLAK\POWER PULSE - PROJE\PLANLAMA\02 - YETKİSİZ KULLANICI - KAYIT VE GİRİŞ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D3846FE-512C-4943-867A-AD9D6BB890A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27467649-6D7F-41C1-94AA-A6CBA5B2EC5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="12090" firstSheet="11" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="2. GEREKSİNİM TAKİP MATRİKSİ" sheetId="18" r:id="rId1"/>
+    <sheet name="2. GEREKSİNİM TAKİP MATRİSİ" sheetId="18" r:id="rId1"/>
     <sheet name="2.1. SİGN IN FORM İÇERİĞİ" sheetId="12" r:id="rId2"/>
     <sheet name="2.1.1. SIGN IN FORM İÇERİĞİ" sheetId="1" r:id="rId3"/>
     <sheet name="2.1.2. SIGN IN FORM İÇERİĞİ -" sheetId="2" r:id="rId4"/>
-    <sheet name="2.2.3.KULLANICI VARLIĞI-SIGN IN" sheetId="13" r:id="rId5"/>
+    <sheet name="2.1.3.KULLANICI VARLIĞI-SIGN IN" sheetId="13" r:id="rId5"/>
     <sheet name="2.3. SIGN UP FORM İÇERİĞİ" sheetId="3" r:id="rId6"/>
     <sheet name="2.3.1. SIGN UP FORM DOĞRULAMA +" sheetId="4" r:id="rId7"/>
     <sheet name="2.3.1.1. BUG RAPORU" sheetId="14" r:id="rId8"/>
@@ -853,9 +853,6 @@
     <t>Yetkisiz Kullanıcı - Kayıt ve Giriş</t>
   </si>
   <si>
-    <t>2. Gereksinim Takip Matriksi</t>
-  </si>
-  <si>
     <t>RTM - 002 [UA - SISU]</t>
   </si>
   <si>
@@ -1241,17 +1238,28 @@
   <si>
     <t>Parola 8 karakter ve harfler ve  rakamlar ve işaretler içerecek şekilde girilir.</t>
   </si>
+  <si>
+    <t>2. Gereksinim Takip Matrisi</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="162"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1969,125 +1977,125 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="33" applyAlignment="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="33" applyAlignment="0"/>
   </cellStyleXfs>
   <cellXfs count="151">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -2096,30 +2104,30 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -2128,112 +2136,112 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
@@ -2242,73 +2250,73 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1"/>
@@ -2832,8 +2840,8 @@
       <c r="A1" s="43" t="s">
         <v>190</v>
       </c>
-      <c r="B1" s="77" t="s">
-        <v>205</v>
+      <c r="B1" s="76" t="s">
+        <v>300</v>
       </c>
       <c r="C1" s="77"/>
       <c r="D1" s="77"/>
@@ -2844,7 +2852,7 @@
         <v>191</v>
       </c>
       <c r="B2" s="77" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C2" s="77"/>
       <c r="F2" s="45" t="s">
@@ -2877,7 +2885,7 @@
         <v>195</v>
       </c>
       <c r="B4" s="78" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C4" s="78"/>
       <c r="F4" s="43" t="s">
@@ -2900,7 +2908,7 @@
         <v>199</v>
       </c>
       <c r="C7" s="65" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D7" s="48" t="s">
         <v>200</v>
@@ -2915,1255 +2923,1255 @@
         <v>203</v>
       </c>
       <c r="H7" s="41" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="63" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="62" t="s">
-        <v>208</v>
+      <c r="A8" s="63" t="s">
+        <v>207</v>
       </c>
       <c r="B8" s="49" t="s">
         <v>145</v>
       </c>
       <c r="C8" s="49" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D8" s="60" t="s">
         <v>180</v>
       </c>
-      <c r="E8" s="69" t="s">
-        <v>218</v>
+      <c r="E8" s="68" t="s">
+        <v>217</v>
       </c>
       <c r="F8" s="49" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G8" s="64" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="H8" s="49" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="58.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="62" t="s">
-        <v>209</v>
+      <c r="A9" s="63" t="s">
+        <v>208</v>
       </c>
       <c r="B9" s="49" t="s">
         <v>145</v>
       </c>
       <c r="C9" s="49" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D9" s="60" t="s">
         <v>180</v>
       </c>
-      <c r="E9" s="69" t="s">
-        <v>218</v>
+      <c r="E9" s="68" t="s">
+        <v>217</v>
       </c>
       <c r="F9" s="49" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G9" s="64" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="H9" s="49" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="60.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="62" t="s">
-        <v>210</v>
+      <c r="A10" s="63" t="s">
+        <v>209</v>
       </c>
       <c r="B10" s="49" t="s">
         <v>145</v>
       </c>
       <c r="C10" s="49" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D10" s="60" t="s">
         <v>180</v>
       </c>
-      <c r="E10" s="69" t="s">
-        <v>218</v>
+      <c r="E10" s="68" t="s">
+        <v>217</v>
       </c>
       <c r="F10" s="49" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G10" s="64" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="H10" s="49" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="82" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="62" t="s">
-        <v>211</v>
+      <c r="A11" s="63" t="s">
+        <v>210</v>
       </c>
       <c r="B11" s="49" t="s">
         <v>93</v>
       </c>
       <c r="C11" s="49" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D11" s="60" t="s">
         <v>180</v>
       </c>
-      <c r="E11" s="69" t="s">
-        <v>218</v>
+      <c r="E11" s="68" t="s">
+        <v>217</v>
       </c>
       <c r="F11" s="49" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G11" s="64" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="H11" s="66" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="64" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A12" s="58" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B12" s="49" t="s">
         <v>93</v>
       </c>
       <c r="C12" s="49" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D12" s="60" t="s">
         <v>180</v>
       </c>
-      <c r="E12" s="69" t="s">
-        <v>218</v>
+      <c r="E12" s="68" t="s">
+        <v>217</v>
       </c>
       <c r="F12" s="49" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G12" s="64" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="H12" s="66" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="65" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A13" s="58" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B13" s="49" t="s">
         <v>145</v>
       </c>
       <c r="C13" s="49" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D13" s="64" t="s">
-        <v>218</v>
-      </c>
-      <c r="E13" s="70" t="s">
+        <v>217</v>
+      </c>
+      <c r="E13" s="69" t="s">
         <v>181</v>
       </c>
       <c r="F13" s="49" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G13" s="64" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="H13" s="66" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="65" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A14" s="63" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B14" s="49" t="s">
         <v>145</v>
       </c>
       <c r="C14" s="49" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D14" s="64" t="s">
-        <v>218</v>
-      </c>
-      <c r="E14" s="70" t="s">
+        <v>217</v>
+      </c>
+      <c r="E14" s="69" t="s">
         <v>182</v>
       </c>
       <c r="F14" s="49" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G14" s="64" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="H14" s="66" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="64.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="63" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B15" s="49" t="s">
         <v>145</v>
       </c>
       <c r="C15" s="49" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D15" s="64" t="s">
-        <v>218</v>
-      </c>
-      <c r="E15" s="70" t="s">
+        <v>217</v>
+      </c>
+      <c r="E15" s="69" t="s">
         <v>183</v>
       </c>
       <c r="F15" s="49" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G15" s="64" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="H15" s="49" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="63" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B16" s="49" t="s">
         <v>145</v>
       </c>
       <c r="C16" s="49" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D16" s="49" t="s">
         <v>184</v>
       </c>
-      <c r="E16" s="69" t="s">
-        <v>218</v>
+      <c r="E16" s="68" t="s">
+        <v>217</v>
       </c>
       <c r="F16" s="49" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G16" s="64" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="H16" s="49" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="68" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="63" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B17" s="49" t="s">
         <v>145</v>
       </c>
       <c r="C17" s="49" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D17" s="49" t="s">
         <v>184</v>
       </c>
-      <c r="E17" s="69" t="s">
-        <v>218</v>
+      <c r="E17" s="68" t="s">
+        <v>217</v>
       </c>
       <c r="F17" s="49" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G17" s="64" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="H17" s="49" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="66.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="63" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B18" s="49" t="s">
         <v>145</v>
       </c>
       <c r="C18" s="49" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D18" s="49" t="s">
         <v>184</v>
       </c>
-      <c r="E18" s="69" t="s">
-        <v>218</v>
+      <c r="E18" s="68" t="s">
+        <v>217</v>
       </c>
       <c r="F18" s="49" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G18" s="64" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="H18" s="49" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="65.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="63" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B19" s="49" t="s">
         <v>145</v>
       </c>
       <c r="C19" s="49" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D19" s="49" t="s">
         <v>184</v>
       </c>
-      <c r="E19" s="69" t="s">
-        <v>218</v>
+      <c r="E19" s="68" t="s">
+        <v>217</v>
       </c>
       <c r="F19" s="49" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G19" s="64" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="H19" s="49" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="85" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="63" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B20" s="49" t="s">
         <v>93</v>
       </c>
       <c r="C20" s="49" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D20" s="49" t="s">
         <v>184</v>
       </c>
-      <c r="E20" s="69" t="s">
-        <v>218</v>
+      <c r="E20" s="68" t="s">
+        <v>217</v>
       </c>
       <c r="F20" s="49" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G20" s="64" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="H20" s="49" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="63" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="63" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B21" s="49" t="s">
         <v>93</v>
       </c>
       <c r="C21" s="49" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D21" s="59" t="s">
         <v>184</v>
       </c>
-      <c r="E21" s="71" t="s">
-        <v>218</v>
+      <c r="E21" s="70" t="s">
+        <v>217</v>
       </c>
       <c r="F21" s="49" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G21" s="64" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="H21" s="49" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="63" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="58" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B22" s="49" t="s">
         <v>145</v>
       </c>
       <c r="C22" s="49" t="s">
-        <v>216</v>
-      </c>
-      <c r="D22" s="68" t="s">
-        <v>218</v>
-      </c>
-      <c r="E22" s="72" t="s">
+        <v>215</v>
+      </c>
+      <c r="D22" s="67" t="s">
+        <v>217</v>
+      </c>
+      <c r="E22" s="71" t="s">
         <v>170</v>
       </c>
       <c r="F22" s="49" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G22" s="64" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="H22" s="49" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="63.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="58" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B23" s="49" t="s">
         <v>145</v>
       </c>
       <c r="C23" s="49" t="s">
-        <v>216</v>
-      </c>
-      <c r="D23" s="68" t="s">
-        <v>218</v>
-      </c>
-      <c r="E23" s="72" t="s">
+        <v>215</v>
+      </c>
+      <c r="D23" s="67" t="s">
+        <v>217</v>
+      </c>
+      <c r="E23" s="71" t="s">
         <v>170</v>
       </c>
       <c r="F23" s="49" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G23" s="64" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="H23" s="49" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="66" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="58" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B24" s="49" t="s">
         <v>145</v>
       </c>
       <c r="C24" s="49" t="s">
-        <v>216</v>
-      </c>
-      <c r="D24" s="68" t="s">
-        <v>218</v>
-      </c>
-      <c r="E24" s="72" t="s">
+        <v>215</v>
+      </c>
+      <c r="D24" s="67" t="s">
+        <v>217</v>
+      </c>
+      <c r="E24" s="71" t="s">
         <v>170</v>
       </c>
       <c r="F24" s="49" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G24" s="64" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="H24" s="49" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="67" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="58" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B25" s="49" t="s">
         <v>145</v>
       </c>
       <c r="C25" s="49" t="s">
-        <v>216</v>
-      </c>
-      <c r="D25" s="68" t="s">
-        <v>218</v>
-      </c>
-      <c r="E25" s="72" t="s">
+        <v>215</v>
+      </c>
+      <c r="D25" s="67" t="s">
+        <v>217</v>
+      </c>
+      <c r="E25" s="71" t="s">
         <v>170</v>
       </c>
       <c r="F25" s="49" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="G25" s="49" t="s">
         <v>186</v>
       </c>
       <c r="H25" s="49" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="69" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="67" t="s">
-        <v>234</v>
+      <c r="A26" s="58" t="s">
+        <v>233</v>
       </c>
       <c r="B26" s="49" t="s">
         <v>145</v>
       </c>
       <c r="C26" s="49" t="s">
-        <v>216</v>
-      </c>
-      <c r="D26" s="68" t="s">
-        <v>218</v>
+        <v>215</v>
+      </c>
+      <c r="D26" s="67" t="s">
+        <v>217</v>
       </c>
       <c r="E26" s="49" t="s">
         <v>172</v>
       </c>
       <c r="F26" s="49" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G26" s="64" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="H26" s="49" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="27" spans="1:8" ht="91.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="67" t="s">
-        <v>235</v>
+      <c r="A27" s="58" t="s">
+        <v>234</v>
       </c>
       <c r="B27" s="49" t="s">
         <v>145</v>
       </c>
       <c r="C27" s="49" t="s">
-        <v>216</v>
-      </c>
-      <c r="D27" s="68" t="s">
-        <v>218</v>
+        <v>215</v>
+      </c>
+      <c r="D27" s="67" t="s">
+        <v>217</v>
       </c>
       <c r="E27" s="49" t="s">
         <v>172</v>
       </c>
       <c r="F27" s="49" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G27" s="64" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="H27" s="49" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="28" spans="1:8" ht="70" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A28" s="58" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B28" s="49" t="s">
         <v>145</v>
       </c>
       <c r="C28" s="49" t="s">
-        <v>216</v>
-      </c>
-      <c r="D28" s="68" t="s">
-        <v>218</v>
+        <v>215</v>
+      </c>
+      <c r="D28" s="67" t="s">
+        <v>217</v>
       </c>
       <c r="E28" s="49" t="s">
         <v>172</v>
       </c>
       <c r="F28" s="49" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G28" s="64" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="H28" s="49" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="29" spans="1:8" ht="97" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A29" s="58" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B29" s="49" t="s">
         <v>145</v>
       </c>
       <c r="C29" s="49" t="s">
-        <v>216</v>
-      </c>
-      <c r="D29" s="68" t="s">
-        <v>218</v>
+        <v>215</v>
+      </c>
+      <c r="D29" s="67" t="s">
+        <v>217</v>
       </c>
       <c r="E29" s="61" t="s">
         <v>185</v>
       </c>
       <c r="F29" s="49" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G29" s="64" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="H29" s="49" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="101" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A30" s="58" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B30" s="49" t="s">
         <v>145</v>
       </c>
       <c r="C30" s="49" t="s">
-        <v>216</v>
-      </c>
-      <c r="D30" s="68" t="s">
-        <v>218</v>
+        <v>215</v>
+      </c>
+      <c r="D30" s="67" t="s">
+        <v>217</v>
       </c>
       <c r="E30" s="61" t="s">
         <v>185</v>
       </c>
       <c r="F30" s="49" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G30" s="64" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="H30" s="49" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="31" spans="1:8" ht="88" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A31" s="58" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B31" s="49" t="s">
         <v>145</v>
       </c>
       <c r="C31" s="49" t="s">
-        <v>216</v>
-      </c>
-      <c r="D31" s="68" t="s">
-        <v>218</v>
+        <v>215</v>
+      </c>
+      <c r="D31" s="67" t="s">
+        <v>217</v>
       </c>
       <c r="E31" s="61" t="s">
         <v>185</v>
       </c>
       <c r="F31" s="49" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G31" s="64" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="H31" s="49" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="32" spans="1:8" ht="95.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A32" s="58" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B32" s="49" t="s">
         <v>145</v>
       </c>
       <c r="C32" s="49" t="s">
-        <v>216</v>
-      </c>
-      <c r="D32" s="68" t="s">
-        <v>218</v>
+        <v>215</v>
+      </c>
+      <c r="D32" s="67" t="s">
+        <v>217</v>
       </c>
       <c r="E32" s="61" t="s">
         <v>185</v>
       </c>
       <c r="F32" s="49" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G32" s="64" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="H32" s="49" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="33" spans="1:8" ht="95.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A33" s="58" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B33" s="49" t="s">
         <v>145</v>
       </c>
       <c r="C33" s="49" t="s">
-        <v>216</v>
-      </c>
-      <c r="D33" s="68" t="s">
-        <v>218</v>
+        <v>215</v>
+      </c>
+      <c r="D33" s="67" t="s">
+        <v>217</v>
       </c>
       <c r="E33" s="61" t="s">
         <v>185</v>
       </c>
       <c r="F33" s="49" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G33" s="64" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="H33" s="49" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="34" spans="1:8" ht="82.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A34" s="58" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B34" s="49" t="s">
         <v>145</v>
       </c>
       <c r="C34" s="49" t="s">
-        <v>216</v>
-      </c>
-      <c r="D34" s="68" t="s">
-        <v>218</v>
+        <v>215</v>
+      </c>
+      <c r="D34" s="67" t="s">
+        <v>217</v>
       </c>
       <c r="E34" s="61" t="s">
         <v>185</v>
       </c>
       <c r="F34" s="49" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G34" s="64" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="H34" s="49" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="35" spans="1:8" ht="109" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="58" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B35" s="49" t="s">
         <v>145</v>
       </c>
       <c r="C35" s="49" t="s">
-        <v>216</v>
-      </c>
-      <c r="D35" s="68" t="s">
-        <v>218</v>
+        <v>215</v>
+      </c>
+      <c r="D35" s="67" t="s">
+        <v>217</v>
       </c>
       <c r="E35" s="61" t="s">
         <v>185</v>
       </c>
       <c r="F35" s="49" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G35" s="64" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="H35" s="49" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="36" spans="1:8" ht="85" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="58" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B36" s="49" t="s">
         <v>145</v>
       </c>
       <c r="C36" s="49" t="s">
-        <v>216</v>
-      </c>
-      <c r="D36" s="68" t="s">
-        <v>218</v>
+        <v>215</v>
+      </c>
+      <c r="D36" s="67" t="s">
+        <v>217</v>
       </c>
       <c r="E36" s="49" t="s">
         <v>173</v>
       </c>
       <c r="F36" s="49" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="G36" s="49" t="s">
         <v>174</v>
       </c>
       <c r="H36" s="49" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="37" spans="1:8" ht="89" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="62" t="s">
-        <v>245</v>
+      <c r="A37" s="63" t="s">
+        <v>244</v>
       </c>
       <c r="B37" s="49" t="s">
         <v>145</v>
       </c>
       <c r="C37" s="49" t="s">
-        <v>216</v>
-      </c>
-      <c r="D37" s="68" t="s">
-        <v>218</v>
+        <v>215</v>
+      </c>
+      <c r="D37" s="67" t="s">
+        <v>217</v>
       </c>
       <c r="E37" s="49" t="s">
         <v>173</v>
       </c>
       <c r="F37" s="49" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="G37" s="49" t="s">
         <v>174</v>
       </c>
       <c r="H37" s="49" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="38" spans="1:8" ht="83" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="62" t="s">
-        <v>246</v>
+      <c r="A38" s="63" t="s">
+        <v>245</v>
       </c>
       <c r="B38" s="49" t="s">
         <v>145</v>
       </c>
       <c r="C38" s="49" t="s">
-        <v>216</v>
-      </c>
-      <c r="D38" s="68" t="s">
-        <v>218</v>
+        <v>215</v>
+      </c>
+      <c r="D38" s="67" t="s">
+        <v>217</v>
       </c>
       <c r="E38" s="49" t="s">
         <v>173</v>
       </c>
       <c r="F38" s="49" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="G38" s="49" t="s">
         <v>174</v>
       </c>
       <c r="H38" s="49" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="95" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" s="58" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B39" s="49" t="s">
         <v>145</v>
       </c>
       <c r="C39" s="49" t="s">
-        <v>216</v>
-      </c>
-      <c r="D39" s="68" t="s">
-        <v>218</v>
+        <v>215</v>
+      </c>
+      <c r="D39" s="67" t="s">
+        <v>217</v>
       </c>
       <c r="E39" s="49" t="s">
         <v>173</v>
       </c>
       <c r="F39" s="49" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="G39" s="49" t="s">
         <v>174</v>
       </c>
       <c r="H39" s="49" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="40" spans="1:8" ht="88" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="58" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B40" s="49" t="s">
         <v>145</v>
       </c>
       <c r="C40" s="49" t="s">
-        <v>216</v>
-      </c>
-      <c r="D40" s="68" t="s">
-        <v>218</v>
+        <v>215</v>
+      </c>
+      <c r="D40" s="67" t="s">
+        <v>217</v>
       </c>
       <c r="E40" s="49" t="s">
         <v>173</v>
       </c>
       <c r="F40" s="49" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="G40" s="49" t="s">
         <v>174</v>
       </c>
       <c r="H40" s="49" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="41" spans="1:8" ht="75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="62" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B41" s="49" t="s">
         <v>93</v>
       </c>
       <c r="C41" s="49" t="s">
-        <v>216</v>
-      </c>
-      <c r="D41" s="68" t="s">
-        <v>218</v>
+        <v>215</v>
+      </c>
+      <c r="D41" s="67" t="s">
+        <v>217</v>
       </c>
       <c r="E41" s="49" t="s">
         <v>173</v>
       </c>
       <c r="F41" s="49" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G41" s="64" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="H41" s="49" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="42" spans="1:8" ht="77.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="58" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B42" s="49" t="s">
         <v>145</v>
       </c>
       <c r="C42" s="49" t="s">
-        <v>216</v>
-      </c>
-      <c r="D42" s="68" t="s">
-        <v>218</v>
+        <v>215</v>
+      </c>
+      <c r="D42" s="67" t="s">
+        <v>217</v>
       </c>
       <c r="E42" s="49" t="s">
         <v>175</v>
       </c>
       <c r="F42" s="49" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G42" s="64" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="H42" s="49" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="43" spans="1:8" ht="82.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" s="58" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B43" s="49" t="s">
         <v>145</v>
       </c>
       <c r="C43" s="49" t="s">
-        <v>216</v>
-      </c>
-      <c r="D43" s="68" t="s">
-        <v>218</v>
+        <v>215</v>
+      </c>
+      <c r="D43" s="67" t="s">
+        <v>217</v>
       </c>
       <c r="E43" s="49" t="s">
         <v>175</v>
       </c>
       <c r="F43" s="49" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="G43" s="44" t="s">
         <v>176</v>
       </c>
       <c r="H43" s="49" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="44" spans="1:8" ht="79.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" s="58" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B44" s="49" t="s">
         <v>145</v>
       </c>
       <c r="C44" s="49" t="s">
-        <v>216</v>
-      </c>
-      <c r="D44" s="68" t="s">
-        <v>218</v>
+        <v>215</v>
+      </c>
+      <c r="D44" s="67" t="s">
+        <v>217</v>
       </c>
       <c r="E44" s="49" t="s">
         <v>175</v>
       </c>
       <c r="F44" s="49" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G44" s="64" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="H44" s="49" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="45" spans="1:8" ht="117.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" s="58" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B45" s="49" t="s">
         <v>145</v>
       </c>
       <c r="C45" s="49" t="s">
-        <v>216</v>
-      </c>
-      <c r="D45" s="68" t="s">
-        <v>218</v>
+        <v>215</v>
+      </c>
+      <c r="D45" s="67" t="s">
+        <v>217</v>
       </c>
       <c r="E45" s="44" t="s">
         <v>175</v>
       </c>
       <c r="F45" s="49" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="G45" s="44" t="s">
         <v>179</v>
       </c>
       <c r="H45" s="49" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="46" spans="1:8" ht="69.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" s="63" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B46" s="49" t="s">
         <v>145</v>
       </c>
       <c r="C46" s="49" t="s">
-        <v>216</v>
-      </c>
-      <c r="D46" s="68" t="s">
-        <v>218</v>
+        <v>215</v>
+      </c>
+      <c r="D46" s="67" t="s">
+        <v>217</v>
       </c>
       <c r="E46" s="49" t="s">
         <v>177</v>
       </c>
       <c r="F46" s="49" t="s">
-        <v>250</v>
-      </c>
-      <c r="G46" s="68" t="s">
-        <v>218</v>
+        <v>249</v>
+      </c>
+      <c r="G46" s="67" t="s">
+        <v>217</v>
       </c>
       <c r="H46" s="49" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="47" spans="1:8" ht="81" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" s="63" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B47" s="49" t="s">
         <v>145</v>
       </c>
       <c r="C47" s="49" t="s">
-        <v>216</v>
-      </c>
-      <c r="D47" s="68" t="s">
-        <v>218</v>
+        <v>215</v>
+      </c>
+      <c r="D47" s="67" t="s">
+        <v>217</v>
       </c>
       <c r="E47" s="49" t="s">
         <v>177</v>
       </c>
       <c r="F47" s="49" t="s">
-        <v>250</v>
-      </c>
-      <c r="G47" s="68" t="s">
-        <v>218</v>
+        <v>249</v>
+      </c>
+      <c r="G47" s="67" t="s">
+        <v>217</v>
       </c>
       <c r="H47" s="49" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="48" spans="1:8" ht="97" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A48" s="63" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B48" s="49" t="s">
         <v>145</v>
       </c>
       <c r="C48" s="49" t="s">
-        <v>216</v>
-      </c>
-      <c r="D48" s="68" t="s">
-        <v>218</v>
+        <v>215</v>
+      </c>
+      <c r="D48" s="67" t="s">
+        <v>217</v>
       </c>
       <c r="E48" s="49" t="s">
         <v>177</v>
       </c>
       <c r="F48" s="49" t="s">
-        <v>250</v>
-      </c>
-      <c r="G48" s="68" t="s">
-        <v>218</v>
+        <v>249</v>
+      </c>
+      <c r="G48" s="67" t="s">
+        <v>217</v>
       </c>
       <c r="H48" s="49" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="49" spans="1:8" ht="74" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A49" s="63" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B49" s="49" t="s">
         <v>145</v>
       </c>
       <c r="C49" s="49" t="s">
-        <v>216</v>
-      </c>
-      <c r="D49" s="68" t="s">
-        <v>218</v>
+        <v>215</v>
+      </c>
+      <c r="D49" s="67" t="s">
+        <v>217</v>
       </c>
       <c r="E49" s="49" t="s">
         <v>177</v>
       </c>
       <c r="F49" s="49" t="s">
-        <v>250</v>
-      </c>
-      <c r="G49" s="68" t="s">
-        <v>218</v>
+        <v>249</v>
+      </c>
+      <c r="G49" s="67" t="s">
+        <v>217</v>
       </c>
       <c r="H49" s="49" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="50" spans="1:8" ht="72.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A50" s="63" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B50" s="49" t="s">
         <v>145</v>
       </c>
       <c r="C50" s="49" t="s">
-        <v>216</v>
-      </c>
-      <c r="D50" s="68" t="s">
-        <v>218</v>
+        <v>215</v>
+      </c>
+      <c r="D50" s="67" t="s">
+        <v>217</v>
       </c>
       <c r="E50" s="49" t="s">
         <v>177</v>
       </c>
       <c r="F50" s="49" t="s">
-        <v>250</v>
-      </c>
-      <c r="G50" s="68" t="s">
-        <v>218</v>
+        <v>249</v>
+      </c>
+      <c r="G50" s="67" t="s">
+        <v>217</v>
       </c>
       <c r="H50" s="49" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="51" spans="1:8" ht="92" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A51" s="63" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B51" s="49" t="s">
         <v>145</v>
       </c>
       <c r="C51" s="49" t="s">
-        <v>216</v>
-      </c>
-      <c r="D51" s="68" t="s">
-        <v>218</v>
+        <v>215</v>
+      </c>
+      <c r="D51" s="67" t="s">
+        <v>217</v>
       </c>
       <c r="E51" s="49" t="s">
         <v>177</v>
       </c>
       <c r="F51" s="49" t="s">
-        <v>250</v>
-      </c>
-      <c r="G51" s="68" t="s">
-        <v>218</v>
+        <v>249</v>
+      </c>
+      <c r="G51" s="67" t="s">
+        <v>217</v>
       </c>
       <c r="H51" s="49" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="52" spans="1:8" ht="80" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A52" s="63" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B52" s="49" t="s">
         <v>145</v>
       </c>
       <c r="C52" s="49" t="s">
-        <v>216</v>
-      </c>
-      <c r="D52" s="68" t="s">
-        <v>218</v>
+        <v>215</v>
+      </c>
+      <c r="D52" s="67" t="s">
+        <v>217</v>
       </c>
       <c r="E52" s="49" t="s">
         <v>177</v>
       </c>
       <c r="F52" s="49" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G52" s="64" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="H52" s="49" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="53" spans="1:8" ht="84" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A53" s="63" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B53" s="49" t="s">
         <v>145</v>
       </c>
       <c r="C53" s="49" t="s">
-        <v>216</v>
-      </c>
-      <c r="D53" s="68" t="s">
-        <v>218</v>
+        <v>215</v>
+      </c>
+      <c r="D53" s="67" t="s">
+        <v>217</v>
       </c>
       <c r="E53" s="49" t="s">
         <v>178</v>
       </c>
       <c r="F53" s="49" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="G53" s="49" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="H53" s="49" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="54" spans="1:8" ht="100.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A54" s="63" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B54" s="49" t="s">
         <v>145</v>
       </c>
       <c r="C54" s="49" t="s">
-        <v>216</v>
-      </c>
-      <c r="D54" s="68" t="s">
-        <v>218</v>
+        <v>215</v>
+      </c>
+      <c r="D54" s="67" t="s">
+        <v>217</v>
       </c>
       <c r="E54" s="49" t="s">
         <v>178</v>
       </c>
       <c r="F54" s="49" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="G54" s="49" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="H54" s="49" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="55" spans="1:8" ht="101.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A55" s="63" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B55" s="49" t="s">
         <v>145</v>
       </c>
       <c r="C55" s="49" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D55" s="64" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="E55" s="49" t="s">
         <v>178</v>
       </c>
       <c r="F55" s="49" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="G55" s="49" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="H55" s="49" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.35">
@@ -4201,7 +4209,7 @@
         <v>1</v>
       </c>
       <c r="D1" s="89" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="E1" s="90"/>
       <c r="F1" s="90"/>
@@ -4428,7 +4436,7 @@
       </c>
       <c r="D15" s="103"/>
       <c r="E15" s="37" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="F15" s="104"/>
       <c r="G15" s="105"/>
@@ -4667,7 +4675,7 @@
         <v>4</v>
       </c>
       <c r="B12" s="86" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C12" s="100"/>
       <c r="D12" s="86" t="s">
@@ -4742,7 +4750,7 @@
       </c>
       <c r="D16" s="103"/>
       <c r="E16" s="37" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="F16" s="104"/>
       <c r="G16" s="105"/>
@@ -5017,7 +5025,7 @@
         <v>5</v>
       </c>
       <c r="B16" s="115" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C16" s="115"/>
       <c r="D16" s="115"/>
@@ -5133,7 +5141,7 @@
         <v>91</v>
       </c>
       <c r="B26" s="136" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="C26" s="136"/>
       <c r="D26" s="136"/>
@@ -5219,7 +5227,7 @@
         <v>1</v>
       </c>
       <c r="D1" s="89" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="E1" s="138"/>
       <c r="F1" s="138"/>
@@ -5434,7 +5442,7 @@
       </c>
       <c r="D15" s="103"/>
       <c r="E15" s="37" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="F15" s="104"/>
       <c r="G15" s="105"/>
@@ -5637,7 +5645,7 @@
       <c r="H10" s="56"/>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A11" s="73" t="s">
+      <c r="A11" s="72" t="s">
         <v>89</v>
       </c>
       <c r="B11" s="55"/>
@@ -5805,7 +5813,7 @@
       <c r="H24" s="54"/>
     </row>
     <row r="25" spans="1:8" ht="277.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="74" t="s">
+      <c r="A25" s="73" t="s">
         <v>90</v>
       </c>
       <c r="B25" s="119"/>
@@ -5817,11 +5825,11 @@
       <c r="H25" s="121"/>
     </row>
     <row r="26" spans="1:8" ht="243.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="75" t="s">
+      <c r="A26" s="74" t="s">
         <v>91</v>
       </c>
       <c r="B26" s="141" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="C26" s="142"/>
       <c r="D26" s="142"/>
@@ -5968,7 +5976,7 @@
         <v>86</v>
       </c>
       <c r="B5" s="115" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C5" s="115"/>
       <c r="D5" s="115"/>
@@ -5982,7 +5990,7 @@
         <v>87</v>
       </c>
       <c r="B6" s="115" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="C6" s="115"/>
       <c r="D6" s="115"/>
@@ -6042,7 +6050,7 @@
       <c r="H10" s="56"/>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A11" s="73" t="s">
+      <c r="A11" s="72" t="s">
         <v>89</v>
       </c>
       <c r="B11" s="55"/>
@@ -6058,7 +6066,7 @@
         <v>1</v>
       </c>
       <c r="B12" s="119" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="C12" s="120"/>
       <c r="D12" s="120"/>
@@ -6104,7 +6112,7 @@
       <c r="H15" s="121"/>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A16" s="73" t="s">
+      <c r="A16" s="72" t="s">
         <v>137</v>
       </c>
       <c r="B16" s="55"/>
@@ -6151,7 +6159,7 @@
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A20" s="140" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B20" s="122"/>
       <c r="C20" s="122"/>
@@ -6198,7 +6206,7 @@
       <c r="H23" s="54"/>
     </row>
     <row r="24" spans="1:8" ht="301" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="74" t="s">
+      <c r="A24" s="73" t="s">
         <v>90</v>
       </c>
       <c r="B24" s="119" t="e" vm="1">
@@ -6212,11 +6220,11 @@
       <c r="H24" s="121"/>
     </row>
     <row r="25" spans="1:8" ht="172" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="75" t="s">
+      <c r="A25" s="74" t="s">
         <v>91</v>
       </c>
       <c r="B25" s="141" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="C25" s="142"/>
       <c r="D25" s="142"/>
@@ -6522,7 +6530,7 @@
       </c>
       <c r="D15" s="103"/>
       <c r="E15" s="37" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="F15" s="104"/>
       <c r="G15" s="105"/>
@@ -6698,7 +6706,7 @@
         <v>77</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="48.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -6718,7 +6726,7 @@
         <v>77</v>
       </c>
       <c r="H9" s="9" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.35">
@@ -6738,7 +6746,7 @@
         <v>77</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
@@ -6799,7 +6807,7 @@
       </c>
       <c r="D15" s="103"/>
       <c r="E15" s="37" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="F15" s="104"/>
       <c r="G15" s="105"/>
@@ -6857,7 +6865,7 @@
         <v>78</v>
       </c>
       <c r="B1" s="42" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="C1" s="117"/>
       <c r="D1" s="135"/>
@@ -6928,7 +6936,7 @@
         <v>86</v>
       </c>
       <c r="B5" s="115" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C5" s="115"/>
       <c r="D5" s="115"/>
@@ -6942,7 +6950,7 @@
         <v>87</v>
       </c>
       <c r="B6" s="115" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C6" s="115"/>
       <c r="D6" s="115"/>
@@ -6953,7 +6961,7 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" s="119" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B7" s="122"/>
       <c r="C7" s="122"/>
@@ -7055,7 +7063,7 @@
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" s="116" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B15" s="116"/>
       <c r="C15" s="116"/>
@@ -7099,7 +7107,7 @@
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A19" s="116" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B19" s="116"/>
       <c r="C19" s="116"/>
@@ -7142,7 +7150,7 @@
       <c r="H22" s="115"/>
     </row>
     <row r="23" spans="1:8" ht="276.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="74" t="s">
+      <c r="A23" s="73" t="s">
         <v>90</v>
       </c>
       <c r="B23" s="115" t="e" vm="2">
@@ -7239,7 +7247,7 @@
         <v>78</v>
       </c>
       <c r="B1" s="51" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="C1" s="117"/>
       <c r="D1" s="135"/>
@@ -7310,7 +7318,7 @@
         <v>86</v>
       </c>
       <c r="B5" s="115" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C5" s="115"/>
       <c r="D5" s="115"/>
@@ -7324,7 +7332,7 @@
         <v>87</v>
       </c>
       <c r="B6" s="115" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C6" s="115"/>
       <c r="D6" s="115"/>
@@ -7335,7 +7343,7 @@
     </row>
     <row r="7" spans="1:9" ht="33" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="146" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B7" s="147"/>
       <c r="C7" s="147"/>
@@ -7402,7 +7410,7 @@
         <v>1</v>
       </c>
       <c r="B12" s="115" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C12" s="115"/>
       <c r="D12" s="115"/>
@@ -7436,7 +7444,7 @@
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" s="116" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B15" s="116"/>
       <c r="C15" s="116"/>
@@ -7480,7 +7488,7 @@
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A19" s="116" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B19" s="116"/>
       <c r="C19" s="116"/>
@@ -7492,7 +7500,7 @@
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A20" s="115" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B20" s="115"/>
       <c r="C20" s="115"/>
@@ -7523,7 +7531,7 @@
       <c r="H22" s="115"/>
     </row>
     <row r="23" spans="1:8" ht="239" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="74" t="s">
+      <c r="A23" s="73" t="s">
         <v>90</v>
       </c>
       <c r="B23" s="115"/>
@@ -7633,7 +7641,7 @@
       <c r="A3" s="30" t="s">
         <v>26</v>
       </c>
-      <c r="B3" s="76">
+      <c r="B3" s="75">
         <v>46222</v>
       </c>
       <c r="C3" s="25"/>
@@ -7794,7 +7802,7 @@
         <v>78</v>
       </c>
       <c r="B1" s="51" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="C1" s="117"/>
       <c r="D1" s="135"/>
@@ -7865,7 +7873,7 @@
         <v>86</v>
       </c>
       <c r="B5" s="115" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C5" s="115"/>
       <c r="D5" s="115"/>
@@ -7879,7 +7887,7 @@
         <v>87</v>
       </c>
       <c r="B6" s="115" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C6" s="115"/>
       <c r="D6" s="115"/>
@@ -7890,7 +7898,7 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" s="119" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B7" s="122"/>
       <c r="C7" s="122"/>
@@ -7957,7 +7965,7 @@
         <v>1</v>
       </c>
       <c r="B12" s="115" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="C12" s="115"/>
       <c r="D12" s="115"/>
@@ -8009,7 +8017,7 @@
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A17" s="116" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B17" s="116"/>
       <c r="C17" s="116"/>
@@ -8053,7 +8061,7 @@
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A21" s="116" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B21" s="116"/>
       <c r="C21" s="116"/>
@@ -8096,7 +8104,7 @@
       <c r="H24" s="115"/>
     </row>
     <row r="25" spans="1:8" ht="281.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="74" t="s">
+      <c r="A25" s="73" t="s">
         <v>90</v>
       </c>
       <c r="B25" s="115" t="e" vm="3">
@@ -8391,7 +8399,7 @@
       </c>
       <c r="D15" s="103"/>
       <c r="E15" s="37" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="F15" s="104"/>
       <c r="G15" s="105"/>
@@ -8671,7 +8679,7 @@
       </c>
       <c r="D15" s="103"/>
       <c r="E15" s="37" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="F15" s="104"/>
       <c r="G15" s="105"/>
@@ -8745,7 +8753,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="92" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C2" s="93"/>
       <c r="D2" s="5" t="s">
@@ -8934,7 +8942,7 @@
       </c>
       <c r="D15" s="103"/>
       <c r="E15" s="37" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="F15" s="104"/>
       <c r="G15" s="105"/>
@@ -9006,7 +9014,7 @@
     </row>
     <row r="3" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A3" s="109" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B3" s="109"/>
       <c r="C3" s="16"/>
@@ -9414,7 +9422,7 @@
       </c>
       <c r="D15" s="103"/>
       <c r="E15" s="37" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="F15" s="104"/>
       <c r="G15" s="105"/>
@@ -9540,7 +9548,7 @@
         <v>86</v>
       </c>
       <c r="B5" s="115" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="C5" s="115"/>
       <c r="D5" s="115"/>
@@ -10107,7 +10115,7 @@
       </c>
       <c r="D16" s="103"/>
       <c r="E16" s="37" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="F16" s="104"/>
       <c r="G16" s="105"/>

</xml_diff>